<commit_message>
fix: correct tourism provenance metadata
</commit_message>
<xml_diff>
--- a/data/final/dataset_maitre_trends_tourisme_afrique.xlsx
+++ b/data/final/dataset_maitre_trends_tourisme_afrique.xlsx
@@ -26013,8 +26013,10 @@
       <x:c r="F511" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G511" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G511" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H511" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26040,11 +26042,15 @@
       <x:c r="O511" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P511" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q511" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P511" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q511" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="512">
@@ -26066,8 +26072,10 @@
       <x:c r="F512" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G512" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G512" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H512" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26093,11 +26101,15 @@
       <x:c r="O512" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P512" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q512" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P512" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q512" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="513">
@@ -26119,8 +26131,10 @@
       <x:c r="F513" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G513" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G513" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H513" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26146,11 +26160,15 @@
       <x:c r="O513" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P513" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q513" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P513" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q513" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="514">
@@ -26172,8 +26190,10 @@
       <x:c r="F514" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G514" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G514" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H514" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26199,11 +26219,15 @@
       <x:c r="O514" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P514" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q514" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P514" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q514" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="515">
@@ -26225,8 +26249,10 @@
       <x:c r="F515" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G515" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G515" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H515" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26252,11 +26278,15 @@
       <x:c r="O515" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P515" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q515" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P515" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q515" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="516">
@@ -26278,8 +26308,10 @@
       <x:c r="F516" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G516" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G516" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H516" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26305,11 +26337,15 @@
       <x:c r="O516" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P516" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q516" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P516" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q516" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="517">
@@ -26331,8 +26367,10 @@
       <x:c r="F517" s="9" t="str">
         <x:v>Europe</x:v>
       </x:c>
-      <x:c r="G517" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G517" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">regional_aggregate</x:t>
+        </x:is>
       </x:c>
       <x:c r="H517" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -26358,11 +26396,15 @@
       <x:c r="O517" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P517" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q517" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P517" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q517" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Groupe régional publié par la source ; composition exacte du groupe à vérifier. Ne pas ventiler en pays et ne pas fusionner automatiquement avec d'autres agrégats scandinaves.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="518">
@@ -28264,11 +28306,15 @@
       <x:c r="O553" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P553" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q553" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P553" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q553" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="554">
@@ -28315,11 +28361,15 @@
       <x:c r="O554" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P554" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q554" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P554" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q554" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="555">
@@ -28631,11 +28681,15 @@
       <x:c r="O560" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P560" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q560" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P560" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q560" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="561">
@@ -28682,11 +28736,15 @@
       <x:c r="O561" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P561" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q561" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P561" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q561" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="562">
@@ -28998,11 +29056,15 @@
       <x:c r="O567" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P567" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q567" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P567" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q567" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="568">
@@ -29049,11 +29111,15 @@
       <x:c r="O568" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P568" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q568" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P568" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q568" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="569">
@@ -29365,11 +29431,15 @@
       <x:c r="O574" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P574" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q574" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P574" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q574" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="575">
@@ -29416,11 +29486,15 @@
       <x:c r="O575" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P575" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q575" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P575" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q575" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="576">
@@ -29732,11 +29806,15 @@
       <x:c r="O581" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P581" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q581" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P581" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q581" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="582">
@@ -29783,11 +29861,15 @@
       <x:c r="O582" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P582" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q582" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P582" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q582" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="583">
@@ -30099,11 +30181,15 @@
       <x:c r="O588" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P588" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q588" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P588" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q588" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="589">
@@ -30150,11 +30236,15 @@
       <x:c r="O589" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P589" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q589" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P589" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q589" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="590">
@@ -30466,11 +30556,15 @@
       <x:c r="O595" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P595" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q595" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P595" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q595" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="596">
@@ -30517,11 +30611,15 @@
       <x:c r="O596" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P596" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q596" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P596" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q596" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="597">
@@ -30833,11 +30931,15 @@
       <x:c r="O602" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P602" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q602" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P602" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q602" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="603">
@@ -30884,11 +30986,15 @@
       <x:c r="O603" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P603" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q603" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P603" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q603" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="604">
@@ -31200,11 +31306,15 @@
       <x:c r="O609" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P609" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q609" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P609" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q609" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="610">
@@ -31251,11 +31361,15 @@
       <x:c r="O610" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P610" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q610" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P610" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q610" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="611">
@@ -32680,11 +32794,15 @@
       <x:c r="O637" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P637" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q637" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P637" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q637" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="638">
@@ -32731,11 +32849,15 @@
       <x:c r="O638" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P638" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q638" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P638" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q638" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="639">
@@ -33047,11 +33169,15 @@
       <x:c r="O644" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P644" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q644" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P644" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q644" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="645">
@@ -33098,11 +33224,15 @@
       <x:c r="O645" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P645" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q645" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P645" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q645" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="646">
@@ -33414,11 +33544,15 @@
       <x:c r="O651" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P651" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q651" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P651" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q651" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="652">
@@ -33465,11 +33599,15 @@
       <x:c r="O652" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P652" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q652" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P652" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q652" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="653">
@@ -33781,11 +33919,15 @@
       <x:c r="O658" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P658" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q658" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P658" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q658" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="659">
@@ -33832,11 +33974,15 @@
       <x:c r="O659" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P659" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q659" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P659" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q659" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="660">
@@ -34519,11 +34665,15 @@
       <x:c r="O672" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P672" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q672" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P672" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q672" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="673">
@@ -34570,11 +34720,15 @@
       <x:c r="O673" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P673" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q673" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P673" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q673" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="674">
@@ -35628,11 +35782,15 @@
       <x:c r="O693" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P693" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q693" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P693" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q693" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="694">
@@ -35679,11 +35837,15 @@
       <x:c r="O694" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P694" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q694" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P694" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q694" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="695">
@@ -35995,11 +36157,15 @@
       <x:c r="O700" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P700" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q700" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P700" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q700" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="701">
@@ -36046,11 +36212,15 @@
       <x:c r="O701" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P701" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q701" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P701" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q701" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="702">
@@ -37104,11 +37274,15 @@
       <x:c r="O721" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P721" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q721" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P721" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q721" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="722">
@@ -37155,11 +37329,15 @@
       <x:c r="O722" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P722" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q722" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P722" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q722" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="723">
@@ -37471,11 +37649,15 @@
       <x:c r="O728" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P728" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q728" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P728" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q728" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="729">
@@ -37522,11 +37704,15 @@
       <x:c r="O729" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P729" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q729" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P729" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q729" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="730">
@@ -37838,11 +38024,15 @@
       <x:c r="O735" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P735" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q735" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P735" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q735" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="736">
@@ -37889,11 +38079,15 @@
       <x:c r="O736" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P736" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q736" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P736" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q736" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="737">
@@ -38205,11 +38399,15 @@
       <x:c r="O742" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P742" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q742" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P742" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q742" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="743">
@@ -38256,11 +38454,15 @@
       <x:c r="O743" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P743" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q743" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P743" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q743" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="744">
@@ -38572,11 +38774,15 @@
       <x:c r="O749" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P749" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q749" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P749" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q749" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="750">
@@ -38623,11 +38829,15 @@
       <x:c r="O750" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P750" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q750" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P750" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q750" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="751">
@@ -38939,11 +39149,15 @@
       <x:c r="O756" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P756" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q756" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P756" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q756" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="757">
@@ -38990,11 +39204,15 @@
       <x:c r="O757" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P757" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q757" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P757" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q757" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="758">
@@ -39306,11 +39524,15 @@
       <x:c r="O763" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P763" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q763" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P763" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q763" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="764">
@@ -39357,11 +39579,15 @@
       <x:c r="O764" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P764" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q764" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P764" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q764" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="765">
@@ -39673,11 +39899,15 @@
       <x:c r="O770" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P770" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q770" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P770" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q770" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="771">
@@ -39724,11 +39954,15 @@
       <x:c r="O771" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P771" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q771" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P771" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q771" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="772">
@@ -40040,11 +40274,15 @@
       <x:c r="O777" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P777" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q777" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P777" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q777" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="778">
@@ -40091,11 +40329,15 @@
       <x:c r="O778" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P778" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q778" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P778" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q778" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="779">
@@ -40407,11 +40649,15 @@
       <x:c r="O784" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P784" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q784" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P784" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q784" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="785">
@@ -40458,11 +40704,15 @@
       <x:c r="O785" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P785" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q785" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P785" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q785" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="786">
@@ -40774,11 +41024,15 @@
       <x:c r="O791" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P791" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q791" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P791" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q791" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="792">
@@ -40825,11 +41079,15 @@
       <x:c r="O792" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P792" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q792" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P792" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q792" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="793">
@@ -41141,11 +41399,15 @@
       <x:c r="O798" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P798" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q798" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P798" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q798" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="799">
@@ -41192,11 +41454,15 @@
       <x:c r="O799" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P799" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q799" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P799" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q799" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="800">
@@ -41508,11 +41774,15 @@
       <x:c r="O805" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P805" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q805" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P805" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q805" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="806">
@@ -41559,11 +41829,15 @@
       <x:c r="O806" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P806" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q806" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P806" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q806" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="807">
@@ -41875,11 +42149,15 @@
       <x:c r="O812" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P812" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q812" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P812" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q812" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="813">
@@ -41926,11 +42204,15 @@
       <x:c r="O813" s="9" t="str">
         <x:v>tunisie_provenance_touristique_2017_2023_ONTT.xlsx</x:v>
       </x:c>
-      <x:c r="P813" s="9" t="str">
-        <x:v>exact_country</x:v>
-      </x:c>
-      <x:c r="Q813" s="9" t="str">
-        <x:v>Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers.</x:v>
+      <x:c r="P813" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="Q813" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Absence d'une nationalité publiée ≠ zéro; TRE non fusionnés avec touristes étrangers. Valeur absente du dataset harmonisé ; cause de l'absence non vérifiée dans la source originale. Ne pas interpréter comme zéro.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="814">
@@ -45185,8 +45467,10 @@
       <x:c r="F875" s="9" t="str">
         <x:v>Other / institutional</x:v>
       </x:c>
-      <x:c r="G875" s="9" t="str">
-        <x:v>country</x:v>
+      <x:c r="G875" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">institutional_category</x:t>
+        </x:is>
       </x:c>
       <x:c r="H875" s="9" t="str">
         <x:v>tourist_origin</x:v>
@@ -45215,8 +45499,10 @@
       <x:c r="P875" s="9" t="str">
         <x:v>exact_top30</x:v>
       </x:c>
-      <x:c r="Q875" s="9" t="str">
-        <x:v>Rang officiel dans le Top 30: 22. La table n'est pas exhaustive de tous les marchés.</x:v>
+      <x:c r="Q875" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rang officiel dans le Top 30: 22. La table n'est pas exhaustive de tous les marchés. Catégorie institutionnelle publiée dans le Top 30 ; ne pas interpréter comme un pays. Définition statistique exacte à vérifier dans la source originale.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="876">
@@ -63853,8 +64139,10 @@
       <x:c r="J7" s="9" t="n">
         <x:v>371</x:v>
       </x:c>
-      <x:c r="K7" s="9" t="str">
-        <x:v>exact_country, exact_diaspora</x:v>
+      <x:c r="K7" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">exact_aggregate, exact_country, exact_diaspora, missing_unverified</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -63993,8 +64281,10 @@
       <x:c r="B8" s="9" t="str">
         <x:v>Niveau statistique</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="str">
-        <x:v>destination_total, country, regional_aggregate, diaspora…</x:v>
+      <x:c r="C8" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">destination_total, country, regional_aggregate, aggregate_total, diaspora, institutional_category. Catégories institutionnelles et agrégées distinctes des pays ; Reunion Island reste country comme marché distinct, sans fusion avec France.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -64059,8 +64349,10 @@
       <x:c r="B14" s="9" t="str">
         <x:v>Producteur/source</x:v>
       </x:c>
-      <x:c r="C14" s="9" t="str">
-        <x:v>World Bank WDI, ONTT, Stats SA…</x:v>
+      <x:c r="C14" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Producteur/source conservé. Égypte–États-Unis : User-provided source file inchangé ; attribution CAPMAS historique non vérifiable avec les pièces présentes dans le dépôt.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -64092,8 +64384,10 @@
       <x:c r="B17" s="9" t="str">
         <x:v>Garde-fou comparatif</x:v>
       </x:c>
-      <x:c r="C17" s="9" t="str">
-        <x:v>Ne jamais ignorer dans le dashboard</x:v>
+      <x:c r="C17" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">missing_unverified : valeur absente du dataset harmonisé, cause non vérifiée dans la source originale ; ne pas assimiler à missing_in_source ni à zéro. Les autres drapeaux restent conservés.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -64148,8 +64442,10 @@
       <x:c r="A4" s="9" t="str">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="9" t="str">
-        <x:v>Aucune donnée manquante n'est remplacée par zéro.</x:v>
+      <x:c r="B4" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Aucune donnée manquante n'est remplacée par zéro. Les 60 absences tunisiennes 2017–2018 portent missing_unverified : cause dans la source non vérifiée.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -64164,24 +64460,30 @@
       <x:c r="A6" s="9" t="str">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="9" t="str">
-        <x:v>Égypte: USA exact + parts régionales 2019; pas de Top pays complet.</x:v>
+      <x:c r="B6" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Égypte: USA exact + parts régionales 2019; pas de Top pays complet. Attribution CAPMAS historique : liaison aux dix observations USA non vérifiable avec les pièces du dépôt ; source_name reste User-provided source file.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="9" t="str">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B7" s="9" t="str">
-        <x:v>Kenya / Maurice / Afrique du Sud: Top 30 / 7 marchés / panel 18 restent explicitement non exhaustifs.</x:v>
+      <x:c r="B7" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Kenya / Maurice / Afrique du Sud: Top 30 / 7 marchés / panel 18 restent explicitement non exhaustifs. Kenya : ONU reste dans le Top 30, en institutional_category. Maurice : Reunion Island reste country, marché distinct sans fusion avec France.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="9" t="str">
-        <x:v>MRE/TRE restent diaspora; Maghreb/Scandinavie/groupes régionaux ne deviennent jamais des pays.</x:v>
+      <x:c r="B8" s="9" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MRE/TRE restent diaspora; Maghreb/Scandinavie/groupes régionaux ne deviennent jamais des pays. Tunisie : les 7 lignes Scandinaves deviennent regional_aggregate / exact_aggregate ; composition exacte à vérifier, sans ventilation ni fusion automatique.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="9">

</xml_diff>